<commit_message>
feat: scale responsibilities and portal operations
</commit_message>
<xml_diff>
--- a/public/Inserate-Studio-Adressimport-Vorlage.xlsx
+++ b/public/Inserate-Studio-Adressimport-Vorlage.xlsx
@@ -542,7 +542,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Fabian&amp;Pascal Inseratestudio · Adressimport</x:v>
+        <x:v>Inserate Studio · Adressimport</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -561,7 +561,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Eine Zeile je Grundstück. Pflichtfelder: Benutzer, Straße, PLZ und Ort. Grundstücksfläche und Preise bitte als Zahlen ohne Einheiten eintragen.</x:v>
+        <x:v>Eine Zeile je Grundstück. Pflichtfelder: Mitarbeiter, Straße, PLZ und Ort. Grundstücksfläche und Preise bitte als Zahlen ohne Einheiten eintragen.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -580,7 +580,7 @@
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:v>Benutzer</x:v>
+        <x:v>Mitarbeiter</x:v>
       </x:c>
       <x:c r="B4" s="17" t="str">
         <x:v>Projektname</x:v>
@@ -627,7 +627,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="30" t="str">
-        <x:v>Fabian</x:v>
+        <x:v>vertrieb@example.de</x:v>
       </x:c>
       <x:c r="B5" s="31" t="str">
         <x:v>Schulzendorf · Beispielgrundstück</x:v>
@@ -2358,11 +2358,6 @@
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
-  <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="A5:A104">
-      <x:formula1>"Fabian,Pascal"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>